<commit_message>
ingesta: snapshot 2026-09-13 18:29 UTC
</commit_message>
<xml_diff>
--- a/data_lake/datos_diarios_preliminares/dt=2026-09-13/CORDOBA_SEP26.xlsx
+++ b/data_lake/datos_diarios_preliminares/dt=2026-09-13/CORDOBA_SEP26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F217A4CD-FA8F-470A-9486-9616FFF47FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2A36A83-6FA2-42D9-A84D-CA9A40E805D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
   </bookViews>
@@ -9993,7 +9993,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>-1</c:v>
@@ -19954,7 +19954,9 @@
       <c r="O3" s="25">
         <v>0</v>
       </c>
-      <c r="P3" s="25"/>
+      <c r="P3" s="25">
+        <v>0</v>
+      </c>
       <c r="Q3" s="25"/>
       <c r="R3" s="25"/>
       <c r="S3" s="25"/>
@@ -20028,7 +20030,9 @@
       <c r="O4" s="25">
         <v>0</v>
       </c>
-      <c r="P4" s="25"/>
+      <c r="P4" s="25">
+        <v>0</v>
+      </c>
       <c r="Q4" s="25"/>
       <c r="R4" s="25"/>
       <c r="S4" s="25"/>
@@ -20102,7 +20106,9 @@
       <c r="O5" s="25">
         <v>0</v>
       </c>
-      <c r="P5" s="25"/>
+      <c r="P5" s="25">
+        <v>0</v>
+      </c>
       <c r="Q5" s="25"/>
       <c r="R5" s="25"/>
       <c r="S5" s="25"/>
@@ -20176,7 +20182,9 @@
       <c r="O6" s="25">
         <v>0</v>
       </c>
-      <c r="P6" s="25"/>
+      <c r="P6" s="25">
+        <v>0</v>
+      </c>
       <c r="Q6" s="25"/>
       <c r="R6" s="25"/>
       <c r="S6" s="25"/>
@@ -20354,7 +20362,9 @@
       <c r="O9" s="25">
         <v>0</v>
       </c>
-      <c r="P9" s="25"/>
+      <c r="P9" s="25">
+        <v>0</v>
+      </c>
       <c r="Q9" s="25"/>
       <c r="R9" s="25"/>
       <c r="S9" s="25"/>
@@ -20478,7 +20488,9 @@
       <c r="O11" s="25">
         <v>0</v>
       </c>
-      <c r="P11" s="25"/>
+      <c r="P11" s="25">
+        <v>0</v>
+      </c>
       <c r="Q11" s="25"/>
       <c r="R11" s="25"/>
       <c r="S11" s="25"/>
@@ -20552,7 +20564,9 @@
       <c r="O12" s="25">
         <v>0</v>
       </c>
-      <c r="P12" s="25"/>
+      <c r="P12" s="25">
+        <v>0</v>
+      </c>
       <c r="Q12" s="25"/>
       <c r="R12" s="25"/>
       <c r="S12" s="25"/>
@@ -20626,7 +20640,9 @@
       <c r="O13" s="25">
         <v>0</v>
       </c>
-      <c r="P13" s="25"/>
+      <c r="P13" s="25">
+        <v>0</v>
+      </c>
       <c r="Q13" s="25"/>
       <c r="R13" s="25"/>
       <c r="S13" s="25"/>
@@ -20698,7 +20714,9 @@
       <c r="O14" s="25">
         <v>0</v>
       </c>
-      <c r="P14" s="25"/>
+      <c r="P14" s="25">
+        <v>0</v>
+      </c>
       <c r="Q14" s="25"/>
       <c r="R14" s="25"/>
       <c r="S14" s="25"/>
@@ -20772,7 +20790,9 @@
       <c r="O15" s="25">
         <v>0</v>
       </c>
-      <c r="P15" s="25"/>
+      <c r="P15" s="25">
+        <v>0</v>
+      </c>
       <c r="Q15" s="25"/>
       <c r="R15" s="25"/>
       <c r="S15" s="25"/>
@@ -20948,7 +20968,7 @@
       </c>
       <c r="P19" s="26">
         <f t="shared" si="1"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="26">
         <f t="shared" si="1"/>

</xml_diff>